<commit_message>
Order Only Bug and Week/Date Addition
FS team found a bug in the Order Only members where I did not have the correct text and I hadn't accounted for new rank fields so was never filtering members when I should have been.
Added Week # and Date to form which needs to be manually entered each week for each file.
</commit_message>
<xml_diff>
--- a/test_notebooks_R/print_04_14_2022.xlsx
+++ b/test_notebooks_R/print_04_14_2022.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="539">
-  <si>
-    <t xml:space="preserve">FSC-T</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="531">
+  <si>
+    <t xml:space="preserve">FSC-T (Week 4 - 04_14_2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Amato, Susan</t>
@@ -458,7 +458,7 @@
     <t xml:space="preserve">5x1 Each Donation to Food Pantry</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD</t>
+    <t xml:space="preserve">FSD (Week 4 - 04_14_2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Carpenter, Rachael</t>
@@ -746,7 +746,7 @@
     <t xml:space="preserve">1x1 Large Horseradish Root</t>
   </si>
   <si>
-    <t xml:space="preserve">FSE</t>
+    <t xml:space="preserve">FSE (Week 4 - 04_14_2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Holzum, Nichole</t>
@@ -968,61 +968,46 @@
     <t xml:space="preserve">1x1 Bottle Thyme for Garlic Vinaigrette</t>
   </si>
   <si>
-    <t xml:space="preserve">Duello, Alex</t>
+    <t xml:space="preserve">Garland, Katherine</t>
   </si>
   <si>
     <t xml:space="preserve">Dawson, Jeff</t>
   </si>
   <si>
+    <t xml:space="preserve">🧀[1]1x1 Each Raw Milk Aged Cheddar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">🐄[*]3x64 Ounce Whole MILK-e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Griffin, Barbara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1x1 Each Field to Fire Option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1x1 Pack Salame - Veneto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kinman, Tricia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lai, Austin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peeler, Michelle</t>
+  </si>
+  <si>
     <t xml:space="preserve">1 No Produce - Order Only (even wk)</t>
   </si>
   <si>
-    <t xml:space="preserve">🧀[1]1x1 Each Raw Milk Aged Cheddar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Garland, Katherine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🐄[*]3x64 Ounce Whole MILK-e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1x1 Pack Salame - Veneto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Griffin, Barbara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Horn, maggie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kinman, Tricia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1x1 Each Field to Fire Option</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kelrick, Michael</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Novalis, Christine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lai, Austin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rothgangel, Ella</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peeler, Michelle</t>
-  </si>
-  <si>
     <t xml:space="preserve">2x1 Lb. Radishes - Watermelon</t>
   </si>
   <si>
     <t xml:space="preserve">2x1 Bag Romaine Lettuce - Loose</t>
   </si>
   <si>
-    <t xml:space="preserve">FSG-Thu</t>
+    <t xml:space="preserve">FSG-Thu (Week 4 - 04_14_2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Rainey, Karen</t>
@@ -1085,7 +1070,7 @@
     <t xml:space="preserve">🌱5x1 Pot Pre-ordered Plants</t>
   </si>
   <si>
-    <t xml:space="preserve">FSMini-t</t>
+    <t xml:space="preserve">FSMini-t (Week 4 - 04_14_2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Heidenheimer, Eileen</t>
@@ -1286,7 +1271,7 @@
     <t xml:space="preserve">t- Vanhooser, Sarah</t>
   </si>
   <si>
-    <t xml:space="preserve">KWA</t>
+    <t xml:space="preserve">KWA (Week 4 - 04_14_2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Arbanas, Michael</t>
@@ -1460,7 +1445,7 @@
     <t xml:space="preserve">2x1 Each Granola Bar</t>
   </si>
   <si>
-    <t xml:space="preserve">KWB</t>
+    <t xml:space="preserve">KWB (Week 4 - 04_14_2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Alexander, Sophia</t>
@@ -1487,12 +1472,6 @@
     <t xml:space="preserve">1x1 Bottle RL Chocolate Milk</t>
   </si>
   <si>
-    <t xml:space="preserve">Guevara, Shannon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Graff, Jeff</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hamper, Laura</t>
   </si>
   <si>
@@ -1538,19 +1517,25 @@
     <t xml:space="preserve">Kreienkamp, Charli</t>
   </si>
   <si>
-    <t xml:space="preserve">Nonnenkamp, Donna</t>
+    <t xml:space="preserve">Senne, Jessica</t>
   </si>
   <si>
     <t xml:space="preserve">🐄[*]2x64 Ounce Whole MILK-e</t>
   </si>
   <si>
+    <t xml:space="preserve">1x16 Ounce Cream pint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4x1 Dozen Eggs - BW</t>
+  </si>
+  <si>
     <t xml:space="preserve">Thomas, Ryan</t>
   </si>
   <si>
-    <t xml:space="preserve">4x1 Dozen Eggs - BW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Senne, Jessica</t>
+    <t xml:space="preserve">1x1 Lb. Pork - Chop bone-in CB /lb.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wippermann, Jennifer</t>
   </si>
   <si>
     <t xml:space="preserve">1x12 Oz. Goshen Colombia</t>
@@ -1559,19 +1544,10 @@
     <t xml:space="preserve">1x1 Bag Goshen Guatemala</t>
   </si>
   <si>
-    <t xml:space="preserve">1x16 Ounce Cream pint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1x1 Lb. Pork - Chop bone-in CB /lb.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wippermann, Jennifer</t>
-  </si>
-  <si>
     <t xml:space="preserve">1x1 Tub FF Dish - Cheesy Polenta</t>
   </si>
   <si>
-    <t xml:space="preserve">KWM</t>
+    <t xml:space="preserve">KWM (Week 4 - 04_14_2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Austin, Anne</t>
@@ -5418,37 +5394,37 @@
         <v>319</v>
       </c>
       <c r="B492" t="s">
-        <v>320</v>
+        <v>247</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="s">
         <v>247</v>
       </c>
-      <c r="B493"/>
+      <c r="B493" s="2" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="494">
       <c r="A494" t="s">
+        <v>320</v>
+      </c>
+      <c r="B494" t="s">
         <v>321</v>
-      </c>
-      <c r="B494" s="1" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="s">
         <v>58</v>
       </c>
-      <c r="B495" t="s">
-        <v>247</v>
-      </c>
+      <c r="B495"/>
     </row>
     <row r="496">
       <c r="A496" t="s">
         <v>29</v>
       </c>
-      <c r="B496" s="2" t="s">
-        <v>135</v>
+      <c r="B496" s="1" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="497">
@@ -5456,44 +5432,58 @@
         <v>57</v>
       </c>
       <c r="B497" t="s">
-        <v>323</v>
+        <v>247</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="s">
         <v>12</v>
       </c>
-      <c r="B498"/>
+      <c r="B498" t="s">
+        <v>305</v>
+      </c>
     </row>
     <row r="499">
       <c r="A499" t="s">
         <v>22</v>
       </c>
-      <c r="B499"/>
+      <c r="B499" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="500">
       <c r="A500" t="s">
         <v>252</v>
       </c>
-      <c r="B500"/>
+      <c r="B500" t="s">
+        <v>323</v>
+      </c>
     </row>
     <row r="501">
       <c r="A501" t="s">
         <v>324</v>
       </c>
-      <c r="B501"/>
+      <c r="B501" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="502">
       <c r="A502"/>
-      <c r="B502"/>
+      <c r="B502" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="503">
       <c r="A503"/>
-      <c r="B503"/>
+      <c r="B503" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="504">
       <c r="A504"/>
-      <c r="B504"/>
+      <c r="B504" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="505">
       <c r="A505"/>
@@ -5524,137 +5514,103 @@
         <v>247</v>
       </c>
       <c r="B509" t="s">
-        <v>320</v>
+        <v>247</v>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="s">
-        <v>305</v>
-      </c>
-      <c r="B510"/>
+        <v>29</v>
+      </c>
+      <c r="B510" s="2" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="511">
       <c r="A511" t="s">
-        <v>29</v>
-      </c>
-      <c r="B511" s="1" t="s">
-        <v>327</v>
-      </c>
+        <v>323</v>
+      </c>
+      <c r="B511"/>
     </row>
     <row r="512">
       <c r="A512" t="s">
-        <v>328</v>
-      </c>
-      <c r="B512" t="s">
-        <v>247</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="B512"/>
     </row>
     <row r="513">
       <c r="A513" t="s">
-        <v>12</v>
-      </c>
-      <c r="B513" t="s">
-        <v>29</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B513"/>
     </row>
     <row r="514">
       <c r="A514" t="s">
-        <v>22</v>
-      </c>
-      <c r="B514" t="s">
+        <v>252</v>
+      </c>
+      <c r="B514"/>
+    </row>
+    <row r="515">
+      <c r="A515"/>
+      <c r="B515"/>
+    </row>
+    <row r="516">
+      <c r="A516" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B516"/>
+    </row>
+    <row r="517">
+      <c r="A517" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="515">
-      <c r="A515" t="s">
-        <v>252</v>
-      </c>
-      <c r="B515" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="516">
-      <c r="A516" t="s">
-        <v>15</v>
-      </c>
-      <c r="B516" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="517">
-      <c r="A517"/>
-      <c r="B517" t="s">
-        <v>252</v>
-      </c>
+      <c r="B517"/>
     </row>
     <row r="518">
-      <c r="A518" s="1" t="s">
+      <c r="A518" t="s">
         <v>329</v>
       </c>
       <c r="B518"/>
     </row>
     <row r="519">
       <c r="A519" t="s">
-        <v>320</v>
-      </c>
-      <c r="B519" s="1" t="s">
         <v>330</v>
       </c>
+      <c r="B519"/>
     </row>
     <row r="520">
       <c r="A520"/>
-      <c r="B520" t="s">
-        <v>320</v>
-      </c>
+      <c r="B520"/>
     </row>
     <row r="521">
-      <c r="A521" s="1" t="s">
-        <v>331</v>
-      </c>
+      <c r="A521"/>
       <c r="B521"/>
     </row>
     <row r="522">
-      <c r="A522" t="s">
-        <v>247</v>
-      </c>
-      <c r="B522" s="1" t="s">
-        <v>332</v>
-      </c>
+      <c r="A522"/>
+      <c r="B522"/>
     </row>
     <row r="523">
-      <c r="A523" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B523" t="s">
-        <v>320</v>
-      </c>
+      <c r="A523"/>
+      <c r="B523"/>
     </row>
     <row r="524">
       <c r="A524"/>
       <c r="B524"/>
     </row>
     <row r="525">
-      <c r="A525" s="1" t="s">
-        <v>333</v>
-      </c>
+      <c r="A525"/>
       <c r="B525"/>
     </row>
     <row r="526">
-      <c r="A526" t="s">
-        <v>320</v>
-      </c>
+      <c r="A526"/>
       <c r="B526"/>
     </row>
     <row r="527">
-      <c r="A527" t="s">
-        <v>334</v>
-      </c>
+      <c r="A527"/>
       <c r="B527"/>
     </row>
     <row r="528">
-      <c r="A528" t="s">
-        <v>335</v>
-      </c>
+      <c r="A528"/>
       <c r="B528"/>
     </row>
     <row r="529">
@@ -5755,18 +5711,18 @@
     </row>
     <row r="553">
       <c r="A553" s="1" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="B553" s="1" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="1" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="B554" s="1" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
     </row>
     <row r="555">
@@ -5779,7 +5735,7 @@
     </row>
     <row r="556">
       <c r="A556" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="B556" t="s">
         <v>58</v>
@@ -5793,10 +5749,10 @@
     </row>
     <row r="558">
       <c r="A558" s="1" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B558" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
     </row>
     <row r="559">
@@ -5807,23 +5763,23 @@
     </row>
     <row r="560">
       <c r="A560" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="B560" s="1" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
     </row>
     <row r="561">
       <c r="A561" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="B561" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
     </row>
     <row r="562">
       <c r="A562" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="B562" t="s">
         <v>58</v>
@@ -5839,21 +5795,21 @@
     </row>
     <row r="564">
       <c r="A564" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="B564" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
     </row>
     <row r="565">
       <c r="A565"/>
       <c r="B565" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="1" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="B566" t="s">
         <v>9</v>
@@ -5864,7 +5820,7 @@
         <v>29</v>
       </c>
       <c r="B567" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
     </row>
     <row r="568">
@@ -5872,12 +5828,12 @@
         <v>57</v>
       </c>
       <c r="B568" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="569">
       <c r="A569" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B569"/>
     </row>
@@ -5886,12 +5842,12 @@
         <v>50</v>
       </c>
       <c r="B570" s="1" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
     </row>
     <row r="571">
       <c r="A571" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="B571" t="s">
         <v>309</v>
@@ -5902,7 +5858,7 @@
         <v>217</v>
       </c>
       <c r="B572" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
     </row>
     <row r="573">
@@ -6011,26 +5967,26 @@
     </row>
     <row r="599">
       <c r="A599" s="1" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="B599" s="1" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="1" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="B600" s="1" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
     </row>
     <row r="601">
       <c r="A601" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B601" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="602">
@@ -6062,7 +6018,7 @@
         <v>32</v>
       </c>
       <c r="B605" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
     </row>
     <row r="606">
@@ -6070,7 +6026,7 @@
         <v>91</v>
       </c>
       <c r="B606" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="607">
@@ -6079,18 +6035,18 @@
     </row>
     <row r="608">
       <c r="A608" s="1" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="B608" s="1" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
     <row r="609">
       <c r="A609" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B609" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="610">
@@ -6103,7 +6059,7 @@
     </row>
     <row r="611">
       <c r="A611" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="B611" t="s">
         <v>129</v>
@@ -6111,7 +6067,7 @@
     </row>
     <row r="612">
       <c r="A612" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="B612" t="s">
         <v>29</v>
@@ -6119,10 +6075,10 @@
     </row>
     <row r="613">
       <c r="A613" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="B613" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
     </row>
     <row r="614">
@@ -6136,18 +6092,18 @@
         <v>7</v>
       </c>
       <c r="B615" s="1" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
     </row>
     <row r="616">
       <c r="A616"/>
       <c r="B616" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="617">
       <c r="A617" s="1" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="B617" s="3" t="s">
         <v>69</v>
@@ -6155,10 +6111,10 @@
     </row>
     <row r="618">
       <c r="A618" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B618" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
     </row>
     <row r="619">
@@ -6171,7 +6127,7 @@
     </row>
     <row r="620">
       <c r="A620" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="B620" t="s">
         <v>29</v>
@@ -6182,12 +6138,12 @@
         <v>292</v>
       </c>
       <c r="B621" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
     </row>
     <row r="622">
       <c r="A622" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="B622" t="s">
         <v>243</v>
@@ -6195,27 +6151,27 @@
     </row>
     <row r="623">
       <c r="A623" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="B623"/>
     </row>
     <row r="624">
       <c r="A624" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="B624" s="1" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
     </row>
     <row r="625">
       <c r="A625"/>
       <c r="B625" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="626">
       <c r="A626" s="1" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B626" s="3" t="s">
         <v>95</v>
@@ -6223,10 +6179,10 @@
     </row>
     <row r="627">
       <c r="A627" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B627" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
     </row>
     <row r="628">
@@ -6242,27 +6198,27 @@
         <v>135</v>
       </c>
       <c r="B629" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
     </row>
     <row r="630">
       <c r="A630"/>
       <c r="B630" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="631">
       <c r="A631" s="1" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B631"/>
     </row>
     <row r="632">
       <c r="A632" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B632" s="1" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
     </row>
     <row r="633">
@@ -6270,12 +6226,12 @@
         <v>95</v>
       </c>
       <c r="B633" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="634">
       <c r="A634" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="B634" s="3" t="s">
         <v>95</v>
@@ -6283,10 +6239,10 @@
     </row>
     <row r="635">
       <c r="A635" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="B635" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
     <row r="636">
@@ -6294,12 +6250,12 @@
         <v>90</v>
       </c>
       <c r="B636" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
     </row>
     <row r="637">
       <c r="A637" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B637" t="s">
         <v>48</v>
@@ -6337,26 +6293,26 @@
     </row>
     <row r="645">
       <c r="A645" s="1" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="B645" s="1" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
     </row>
     <row r="646">
       <c r="A646" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="B646" s="1" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="647">
       <c r="A647" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B647" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="648">
@@ -6369,7 +6325,7 @@
     </row>
     <row r="649">
       <c r="A649" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="B649" t="s">
         <v>29</v>
@@ -6377,7 +6333,7 @@
     </row>
     <row r="650">
       <c r="A650" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="B650" t="s">
         <v>65</v>
@@ -6385,10 +6341,10 @@
     </row>
     <row r="651">
       <c r="A651" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="B651" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
     </row>
     <row r="652">
@@ -6399,16 +6355,16 @@
     </row>
     <row r="653">
       <c r="A653" s="1" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="B653"/>
     </row>
     <row r="654">
       <c r="A654" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B654" s="1" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
     </row>
     <row r="655">
@@ -6416,7 +6372,7 @@
         <v>105</v>
       </c>
       <c r="B655" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="656">
@@ -6429,10 +6385,10 @@
     </row>
     <row r="657">
       <c r="A657" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="B657" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
     <row r="658">
@@ -6445,7 +6401,7 @@
     </row>
     <row r="659">
       <c r="A659" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="B659" t="s">
         <v>296</v>
@@ -6454,12 +6410,12 @@
     <row r="660">
       <c r="A660"/>
       <c r="B660" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
     </row>
     <row r="661">
       <c r="A661" s="1" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="B661" t="s">
         <v>147</v>
@@ -6467,29 +6423,29 @@
     </row>
     <row r="662">
       <c r="A662" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B662"/>
     </row>
     <row r="663">
       <c r="A663" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="B663" s="1" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
     <row r="664">
       <c r="A664" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B664" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="665">
       <c r="A665" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="B665" t="s">
         <v>97</v>
@@ -6497,7 +6453,7 @@
     </row>
     <row r="666">
       <c r="A666" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="B666" t="s">
         <v>29</v>
@@ -6506,12 +6462,12 @@
     <row r="667">
       <c r="A667"/>
       <c r="B667" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
     </row>
     <row r="668">
       <c r="A668" s="1" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="B668" t="s">
         <v>264</v>
@@ -6519,7 +6475,7 @@
     </row>
     <row r="669">
       <c r="A669" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B669"/>
     </row>
@@ -6528,18 +6484,18 @@
         <v>135</v>
       </c>
       <c r="B670" s="1" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
     </row>
     <row r="671">
       <c r="A671"/>
       <c r="B671" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="672">
       <c r="A672" s="1" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B672" t="s">
         <v>285</v>
@@ -6547,7 +6503,7 @@
     </row>
     <row r="673">
       <c r="A673" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B673" t="s">
         <v>86</v>
@@ -6555,10 +6511,10 @@
     </row>
     <row r="674">
       <c r="A674" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="B674" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
     </row>
     <row r="675">
@@ -6566,12 +6522,12 @@
         <v>29</v>
       </c>
       <c r="B675" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
     </row>
     <row r="676">
       <c r="A676" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="B676" t="s">
         <v>110</v>
@@ -6579,7 +6535,7 @@
     </row>
     <row r="677">
       <c r="A677" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="B677" t="s">
         <v>205</v>
@@ -6587,27 +6543,27 @@
     </row>
     <row r="678">
       <c r="A678" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="B678"/>
     </row>
     <row r="679">
       <c r="A679"/>
       <c r="B679" s="1" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
     </row>
     <row r="680">
       <c r="A680" s="1" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="B680" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="681">
       <c r="A681" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B681" s="2" t="s">
         <v>135</v>
@@ -6622,20 +6578,20 @@
     <row r="683">
       <c r="A683"/>
       <c r="B683" s="1" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="684">
       <c r="A684" s="1" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="B684" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="685">
       <c r="A685" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B685" s="2" t="s">
         <v>135</v>
@@ -6665,31 +6621,31 @@
     </row>
     <row r="691">
       <c r="A691" s="1" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="B691" s="1" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
     </row>
     <row r="692">
       <c r="A692" s="1" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="B692" s="1" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
     </row>
     <row r="693">
       <c r="A693" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B693" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="694">
       <c r="A694" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B694" t="s">
         <v>56</v>
@@ -6697,7 +6653,7 @@
     </row>
     <row r="695">
       <c r="A695" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="B695" t="s">
         <v>58</v>
@@ -6705,7 +6661,7 @@
     </row>
     <row r="696">
       <c r="A696" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="B696" t="s">
         <v>29</v>
@@ -6727,7 +6683,7 @@
     </row>
     <row r="699">
       <c r="A699" s="1" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="B699" t="s">
         <v>9</v>
@@ -6735,7 +6691,7 @@
     </row>
     <row r="700">
       <c r="A700" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B700" t="s">
         <v>91</v>
@@ -6743,7 +6699,7 @@
     </row>
     <row r="701">
       <c r="A701" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="B701"/>
     </row>
@@ -6752,20 +6708,20 @@
         <v>29</v>
       </c>
       <c r="B702" s="1" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
     </row>
     <row r="703">
       <c r="A703" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="B703" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="704">
       <c r="A704" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="B704" s="2" t="s">
         <v>135</v>
@@ -6780,20 +6736,20 @@
     <row r="706">
       <c r="A706"/>
       <c r="B706" s="1" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
     </row>
     <row r="707">
       <c r="A707" s="1" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="B707" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="708">
       <c r="A708" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B708" s="2" t="s">
         <v>135</v>
@@ -6915,39 +6871,39 @@
     </row>
     <row r="737">
       <c r="A737" s="1" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="B737" s="1" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
     </row>
     <row r="738">
       <c r="A738" s="1" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="B738" s="1" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
     </row>
     <row r="739">
       <c r="A739" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B739" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="740">
       <c r="A740" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B740" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
     </row>
     <row r="741">
       <c r="A741" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="B741" t="s">
         <v>287</v>
@@ -6958,7 +6914,7 @@
         <v>287</v>
       </c>
       <c r="B742" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="743">
@@ -6966,7 +6922,7 @@
         <v>58</v>
       </c>
       <c r="B743" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
     </row>
     <row r="744">
@@ -6974,7 +6930,7 @@
         <v>208</v>
       </c>
       <c r="B744" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
     </row>
     <row r="745">
@@ -6994,28 +6950,28 @@
     <row r="747">
       <c r="A747"/>
       <c r="B747" s="1" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
     </row>
     <row r="748">
       <c r="A748" s="1" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="B748" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="749">
       <c r="A749" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B749" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="750">
       <c r="A750" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="B750" t="s">
         <v>287</v>
@@ -7023,7 +6979,7 @@
     </row>
     <row r="751">
       <c r="A751" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B751" t="s">
         <v>243</v>
@@ -7031,10 +6987,10 @@
     </row>
     <row r="752">
       <c r="A752" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="B752" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
     </row>
     <row r="753">
@@ -7047,10 +7003,10 @@
     </row>
     <row r="754">
       <c r="A754" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="B754" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="755">
@@ -7069,10 +7025,10 @@
     </row>
     <row r="757">
       <c r="A757" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="B757" s="1" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
     </row>
     <row r="758">
@@ -7080,7 +7036,7 @@
         <v>96</v>
       </c>
       <c r="B758" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="759">
@@ -7088,7 +7044,7 @@
         <v>165</v>
       </c>
       <c r="B759" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="760">
@@ -7099,7 +7055,7 @@
     </row>
     <row r="761">
       <c r="A761" s="1" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="B761" t="s">
         <v>58</v>
@@ -7107,23 +7063,23 @@
     </row>
     <row r="762">
       <c r="A762" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B762" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
     </row>
     <row r="763">
       <c r="A763" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="B763" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
     </row>
     <row r="764">
       <c r="A764" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B764" t="s">
         <v>7</v>
@@ -7140,15 +7096,15 @@
         <v>165</v>
       </c>
       <c r="B766" s="1" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
     </row>
     <row r="767">
       <c r="A767" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B767" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="768">
@@ -7156,7 +7112,7 @@
         <v>46</v>
       </c>
       <c r="B768" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
     </row>
     <row r="769">
@@ -7167,7 +7123,7 @@
     </row>
     <row r="770">
       <c r="A770" s="1" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="B770" t="s">
         <v>65</v>
@@ -7175,7 +7131,7 @@
     </row>
     <row r="771">
       <c r="A771" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B771" t="s">
         <v>196</v>
@@ -7183,19 +7139,19 @@
     </row>
     <row r="772">
       <c r="A772" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="B772"/>
     </row>
     <row r="773">
       <c r="A773" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="B773"/>
     </row>
     <row r="774">
       <c r="A774" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="B774"/>
     </row>
@@ -7207,7 +7163,7 @@
     </row>
     <row r="776">
       <c r="A776" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="B776"/>
     </row>
@@ -7237,34 +7193,34 @@
     </row>
     <row r="783">
       <c r="A783" s="1" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="B783" s="1" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
     </row>
     <row r="784">
       <c r="A784" s="1" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
       <c r="B784" s="1" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
     </row>
     <row r="785">
       <c r="A785" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B785" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="786">
       <c r="A786" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="B786" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="787">
@@ -7277,18 +7233,18 @@
     </row>
     <row r="788">
       <c r="A788" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="B788" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
     </row>
     <row r="789">
       <c r="A789" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="B789" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
     </row>
     <row r="790">
@@ -7304,12 +7260,12 @@
         <v>315</v>
       </c>
       <c r="B791" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
     </row>
     <row r="792">
       <c r="A792" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="B792" t="s">
         <v>299</v>
@@ -7324,28 +7280,28 @@
     <row r="794">
       <c r="A794"/>
       <c r="B794" s="1" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
     </row>
     <row r="795">
       <c r="A795" s="1" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="B795" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="796">
       <c r="A796" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B796" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="797">
       <c r="A797" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B797" t="s">
         <v>56</v>
@@ -7353,15 +7309,15 @@
     </row>
     <row r="798">
       <c r="A798" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="B798" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
     </row>
     <row r="799">
       <c r="A799" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
       <c r="B799" t="s">
         <v>109</v>
@@ -7385,7 +7341,7 @@
     </row>
     <row r="802">
       <c r="A802" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="B802" t="s">
         <v>144</v>
@@ -7397,26 +7353,26 @@
     </row>
     <row r="804">
       <c r="A804" s="1" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="B804" s="1" t="s">
-        <v>462</v>
+        <v>457</v>
       </c>
     </row>
     <row r="805">
       <c r="A805" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B805" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="806">
       <c r="A806" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="B806" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="807">
@@ -7424,12 +7380,12 @@
         <v>287</v>
       </c>
       <c r="B807" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
     </row>
     <row r="808">
       <c r="A808" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
       <c r="B808" t="s">
         <v>162</v>
@@ -7437,43 +7393,43 @@
     </row>
     <row r="809">
       <c r="A809" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="B809" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
     </row>
     <row r="810">
       <c r="A810" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B810"/>
     </row>
     <row r="811">
       <c r="A811" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
       <c r="B811" s="1" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
     </row>
     <row r="812">
       <c r="A812"/>
       <c r="B812" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="813">
       <c r="A813" s="1" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
       <c r="B813" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="814">
       <c r="A814" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B814" t="s">
         <v>287</v>
@@ -7484,15 +7440,15 @@
         <v>97</v>
       </c>
       <c r="B815" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
     </row>
     <row r="816">
       <c r="A816" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="B816" t="s">
-        <v>469</v>
+        <v>464</v>
       </c>
     </row>
     <row r="817">
@@ -7505,15 +7461,15 @@
     </row>
     <row r="818">
       <c r="A818" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="B818" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
     </row>
     <row r="819">
       <c r="A819" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="B819"/>
     </row>
@@ -7557,42 +7513,42 @@
     </row>
     <row r="829">
       <c r="A829" s="1" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="B829" s="1" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
     </row>
     <row r="830">
       <c r="A830" s="1" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="B830" s="1" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
     </row>
     <row r="831">
       <c r="A831" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B831" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="832">
       <c r="A832" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B832" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
     </row>
     <row r="833">
       <c r="A833" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="B833" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="834">
@@ -7600,7 +7556,7 @@
         <v>278</v>
       </c>
       <c r="B834" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
     </row>
     <row r="835">
@@ -7616,12 +7572,12 @@
         <v>165</v>
       </c>
       <c r="B836" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
     </row>
     <row r="837">
       <c r="A837" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="B837" t="s">
         <v>49</v>
@@ -7632,7 +7588,7 @@
         <v>70</v>
       </c>
       <c r="B838" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
     </row>
     <row r="839">
@@ -7641,23 +7597,23 @@
     </row>
     <row r="840">
       <c r="A840" s="1" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="B840" s="1" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
     </row>
     <row r="841">
       <c r="A841" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B841" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="842">
       <c r="A842" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="B842" t="s">
         <v>313</v>
@@ -7681,7 +7637,7 @@
     </row>
     <row r="845">
       <c r="A845" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
       <c r="B845" t="s">
         <v>274</v>
@@ -7692,7 +7648,7 @@
         <v>29</v>
       </c>
       <c r="B846" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
     </row>
     <row r="847">
@@ -7700,7 +7656,7 @@
         <v>10</v>
       </c>
       <c r="B847" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
     </row>
     <row r="848">
@@ -7719,7 +7675,7 @@
     </row>
     <row r="850">
       <c r="A850" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="B850"/>
     </row>
@@ -7735,19 +7691,19 @@
     </row>
     <row r="853">
       <c r="A853" s="1" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="B853"/>
     </row>
     <row r="854">
       <c r="A854" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B854"/>
     </row>
     <row r="855">
       <c r="A855" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="B855"/>
     </row>
@@ -7777,7 +7733,7 @@
     </row>
     <row r="860">
       <c r="A860" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="B860"/>
     </row>
@@ -7847,18 +7803,18 @@
     </row>
     <row r="875">
       <c r="A875" s="1" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="B875" s="1" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
     </row>
     <row r="876">
       <c r="A876" s="1" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="B876" s="1" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
     </row>
     <row r="877">
@@ -7871,18 +7827,18 @@
     </row>
     <row r="878">
       <c r="A878" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="B878" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
     </row>
     <row r="879">
       <c r="A879" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="B879" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
     </row>
     <row r="880">
@@ -7890,7 +7846,7 @@
         <v>58</v>
       </c>
       <c r="B880" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
     </row>
     <row r="881">
@@ -7898,15 +7854,15 @@
         <v>48</v>
       </c>
       <c r="B881" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
     </row>
     <row r="882">
       <c r="A882" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="B882" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
     </row>
     <row r="883">
@@ -7917,263 +7873,255 @@
     </row>
     <row r="884">
       <c r="A884" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="B884" s="1" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
     </row>
     <row r="885">
       <c r="A885"/>
       <c r="B885" t="s">
-        <v>320</v>
+        <v>247</v>
       </c>
     </row>
     <row r="886">
       <c r="A886" s="1" t="s">
-        <v>492</v>
-      </c>
-      <c r="B886"/>
+        <v>487</v>
+      </c>
+      <c r="B886" t="s">
+        <v>472</v>
+      </c>
     </row>
     <row r="887">
       <c r="A887" t="s">
-        <v>320</v>
-      </c>
-      <c r="B887" s="1" t="s">
-        <v>493</v>
+        <v>328</v>
+      </c>
+      <c r="B887" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="888">
-      <c r="A888"/>
+      <c r="A888" t="s">
+        <v>488</v>
+      </c>
       <c r="B888" t="s">
-        <v>247</v>
+        <v>489</v>
       </c>
     </row>
     <row r="889">
-      <c r="A889" s="1" t="s">
-        <v>494</v>
+      <c r="A889" t="s">
+        <v>250</v>
       </c>
       <c r="B889" t="s">
-        <v>477</v>
+        <v>29</v>
       </c>
     </row>
     <row r="890">
       <c r="A890" t="s">
-        <v>320</v>
+        <v>166</v>
       </c>
       <c r="B890" t="s">
-        <v>305</v>
+        <v>490</v>
       </c>
     </row>
     <row r="891">
-      <c r="A891" t="s">
-        <v>495</v>
-      </c>
+      <c r="A891"/>
       <c r="B891" t="s">
-        <v>496</v>
+        <v>12</v>
       </c>
     </row>
     <row r="892">
-      <c r="A892" t="s">
-        <v>250</v>
+      <c r="A892" s="1" t="s">
+        <v>491</v>
       </c>
       <c r="B892" t="s">
-        <v>29</v>
+        <v>492</v>
       </c>
     </row>
     <row r="893">
       <c r="A893" t="s">
-        <v>166</v>
+        <v>247</v>
       </c>
       <c r="B893" t="s">
-        <v>497</v>
+        <v>252</v>
       </c>
     </row>
     <row r="894">
-      <c r="A894"/>
-      <c r="B894" t="s">
-        <v>12</v>
-      </c>
+      <c r="A894" t="s">
+        <v>423</v>
+      </c>
+      <c r="B894"/>
     </row>
     <row r="895">
-      <c r="A895" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="B895" t="s">
-        <v>499</v>
+      <c r="A895" t="s">
+        <v>305</v>
+      </c>
+      <c r="B895" s="1" t="s">
+        <v>493</v>
       </c>
     </row>
     <row r="896">
       <c r="A896" t="s">
+        <v>31</v>
+      </c>
+      <c r="B896" t="s">
         <v>247</v>
-      </c>
-      <c r="B896" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="897">
       <c r="A897" t="s">
-        <v>428</v>
-      </c>
-      <c r="B897"/>
+        <v>393</v>
+      </c>
+      <c r="B897" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="898">
       <c r="A898" t="s">
-        <v>305</v>
-      </c>
-      <c r="B898" s="1" t="s">
-        <v>500</v>
+        <v>114</v>
+      </c>
+      <c r="B898" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="899">
       <c r="A899" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B899" t="s">
-        <v>247</v>
+        <v>193</v>
       </c>
     </row>
     <row r="900">
-      <c r="A900" t="s">
-        <v>398</v>
-      </c>
+      <c r="A900"/>
       <c r="B900" t="s">
-        <v>428</v>
+        <v>29</v>
       </c>
     </row>
     <row r="901">
-      <c r="A901" t="s">
-        <v>114</v>
+      <c r="A901" s="1" t="s">
+        <v>494</v>
       </c>
       <c r="B901" t="s">
-        <v>58</v>
+        <v>323</v>
       </c>
     </row>
     <row r="902">
       <c r="A902" t="s">
-        <v>12</v>
+        <v>247</v>
       </c>
       <c r="B902" t="s">
-        <v>193</v>
+        <v>495</v>
       </c>
     </row>
     <row r="903">
-      <c r="A903"/>
+      <c r="A903" t="s">
+        <v>57</v>
+      </c>
       <c r="B903" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="904">
-      <c r="A904" s="1" t="s">
-        <v>501</v>
+      <c r="A904" t="s">
+        <v>496</v>
       </c>
       <c r="B904" t="s">
-        <v>328</v>
+        <v>91</v>
       </c>
     </row>
     <row r="905">
       <c r="A905" t="s">
-        <v>247</v>
-      </c>
-      <c r="B905" t="s">
-        <v>502</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="B905"/>
     </row>
     <row r="906">
       <c r="A906" t="s">
-        <v>57</v>
-      </c>
-      <c r="B906" t="s">
-        <v>22</v>
+        <v>50</v>
+      </c>
+      <c r="B906" s="1" t="s">
+        <v>497</v>
       </c>
     </row>
     <row r="907">
       <c r="A907" t="s">
-        <v>503</v>
+        <v>32</v>
       </c>
       <c r="B907" t="s">
-        <v>91</v>
+        <v>247</v>
       </c>
     </row>
     <row r="908">
       <c r="A908" t="s">
-        <v>259</v>
-      </c>
-      <c r="B908"/>
+        <v>498</v>
+      </c>
+      <c r="B908" t="s">
+        <v>472</v>
+      </c>
     </row>
     <row r="909">
       <c r="A909" t="s">
-        <v>50</v>
-      </c>
-      <c r="B909" s="1" t="s">
-        <v>504</v>
+        <v>7</v>
+      </c>
+      <c r="B909" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="910">
       <c r="A910" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="B910" t="s">
-        <v>247</v>
+        <v>8</v>
       </c>
     </row>
     <row r="911">
       <c r="A911" t="s">
-        <v>505</v>
+        <v>347</v>
       </c>
       <c r="B911" t="s">
-        <v>477</v>
+        <v>323</v>
       </c>
     </row>
     <row r="912">
       <c r="A912" t="s">
-        <v>7</v>
+        <v>499</v>
       </c>
       <c r="B912" t="s">
-        <v>58</v>
+        <v>427</v>
       </c>
     </row>
     <row r="913">
-      <c r="A913" t="s">
-        <v>9</v>
-      </c>
+      <c r="A913"/>
       <c r="B913" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="914">
-      <c r="A914" t="s">
-        <v>352</v>
-      </c>
+      <c r="A914"/>
       <c r="B914" t="s">
-        <v>328</v>
+        <v>252</v>
       </c>
     </row>
     <row r="915">
-      <c r="A915" t="s">
-        <v>506</v>
-      </c>
+      <c r="A915"/>
       <c r="B915" t="s">
-        <v>432</v>
+        <v>110</v>
       </c>
     </row>
     <row r="916">
       <c r="A916"/>
-      <c r="B916" t="s">
-        <v>22</v>
-      </c>
+      <c r="B916"/>
     </row>
     <row r="917">
       <c r="A917"/>
-      <c r="B917" t="s">
-        <v>252</v>
-      </c>
+      <c r="B917"/>
     </row>
     <row r="918">
       <c r="A918"/>
-      <c r="B918" t="s">
-        <v>110</v>
-      </c>
+      <c r="B918"/>
     </row>
     <row r="919">
       <c r="A919"/>
@@ -8185,18 +8133,18 @@
     </row>
     <row r="921">
       <c r="A921" s="1" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="B921" s="1" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
     </row>
     <row r="922">
       <c r="A922" s="1" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
       <c r="B922" s="1" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
     </row>
     <row r="923">
@@ -8204,29 +8152,31 @@
         <v>247</v>
       </c>
       <c r="B923" t="s">
-        <v>320</v>
+        <v>247</v>
       </c>
     </row>
     <row r="924">
       <c r="A924" t="s">
-        <v>509</v>
-      </c>
-      <c r="B924"/>
+        <v>502</v>
+      </c>
+      <c r="B924" t="s">
+        <v>337</v>
+      </c>
     </row>
     <row r="925">
       <c r="A925" t="s">
-        <v>477</v>
-      </c>
-      <c r="B925" s="1" t="s">
-        <v>510</v>
+        <v>472</v>
+      </c>
+      <c r="B925" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="926">
       <c r="A926" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
       <c r="B926" t="s">
-        <v>247</v>
+        <v>129</v>
       </c>
     </row>
     <row r="927">
@@ -8234,7 +8184,7 @@
         <v>22</v>
       </c>
       <c r="B927" t="s">
-        <v>54</v>
+        <v>360</v>
       </c>
     </row>
     <row r="928">
@@ -8242,37 +8192,37 @@
         <v>263</v>
       </c>
       <c r="B928" t="s">
-        <v>29</v>
+        <v>287</v>
       </c>
     </row>
     <row r="929">
       <c r="A929" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B929" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
     </row>
     <row r="930">
       <c r="A930" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="B930" t="s">
-        <v>293</v>
+        <v>368</v>
       </c>
     </row>
     <row r="931">
       <c r="A931"/>
       <c r="B931" t="s">
-        <v>328</v>
+        <v>12</v>
       </c>
     </row>
     <row r="932">
       <c r="A932" s="1" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
       <c r="B932" t="s">
-        <v>431</v>
+        <v>22</v>
       </c>
     </row>
     <row r="933">
@@ -8280,129 +8230,123 @@
         <v>247</v>
       </c>
       <c r="B933" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
     </row>
     <row r="934">
       <c r="A934" t="s">
-        <v>342</v>
-      </c>
-      <c r="B934" t="s">
-        <v>514</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B934"/>
     </row>
     <row r="935">
       <c r="A935" t="s">
-        <v>515</v>
-      </c>
-      <c r="B935" t="s">
-        <v>12</v>
+        <v>29</v>
+      </c>
+      <c r="B935" s="1" t="s">
+        <v>507</v>
       </c>
     </row>
     <row r="936">
       <c r="A936" t="s">
-        <v>129</v>
-      </c>
-      <c r="B936"/>
+        <v>48</v>
+      </c>
+      <c r="B936" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="937">
       <c r="A937" t="s">
-        <v>365</v>
-      </c>
-      <c r="B937"/>
+        <v>293</v>
+      </c>
+      <c r="B937" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="938">
       <c r="A938" t="s">
-        <v>287</v>
-      </c>
-      <c r="B938"/>
+        <v>323</v>
+      </c>
+      <c r="B938" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="939">
       <c r="A939" t="s">
-        <v>29</v>
-      </c>
-      <c r="B939"/>
+        <v>426</v>
+      </c>
+      <c r="B939" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="940">
       <c r="A940" t="s">
-        <v>373</v>
-      </c>
-      <c r="B940"/>
+        <v>508</v>
+      </c>
+      <c r="B940" t="s">
+        <v>313</v>
+      </c>
     </row>
     <row r="941">
       <c r="A941" t="s">
-        <v>12</v>
-      </c>
-      <c r="B941"/>
+        <v>509</v>
+      </c>
+      <c r="B941" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="942">
       <c r="A942" t="s">
-        <v>22</v>
-      </c>
-      <c r="B942"/>
+        <v>12</v>
+      </c>
+      <c r="B942" t="s">
+        <v>510</v>
+      </c>
     </row>
     <row r="943">
-      <c r="A943" t="s">
-        <v>516</v>
-      </c>
-      <c r="B943"/>
+      <c r="A943"/>
+      <c r="B943" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="944">
       <c r="A944"/>
       <c r="B944"/>
     </row>
     <row r="945">
-      <c r="A945" s="1" t="s">
-        <v>517</v>
-      </c>
+      <c r="A945"/>
       <c r="B945"/>
     </row>
     <row r="946">
-      <c r="A946" t="s">
-        <v>247</v>
-      </c>
+      <c r="A946"/>
       <c r="B946"/>
     </row>
     <row r="947">
-      <c r="A947" t="s">
-        <v>137</v>
-      </c>
+      <c r="A947"/>
       <c r="B947"/>
     </row>
     <row r="948">
-      <c r="A948" t="s">
-        <v>428</v>
-      </c>
+      <c r="A948"/>
       <c r="B948"/>
     </row>
     <row r="949">
-      <c r="A949" t="s">
-        <v>54</v>
-      </c>
+      <c r="A949"/>
       <c r="B949"/>
     </row>
     <row r="950">
-      <c r="A950" t="s">
-        <v>313</v>
-      </c>
+      <c r="A950"/>
       <c r="B950"/>
     </row>
     <row r="951">
-      <c r="A951" t="s">
-        <v>31</v>
-      </c>
+      <c r="A951"/>
       <c r="B951"/>
     </row>
     <row r="952">
-      <c r="A952" t="s">
-        <v>518</v>
-      </c>
+      <c r="A952"/>
       <c r="B952"/>
     </row>
     <row r="953">
-      <c r="A953" t="s">
-        <v>252</v>
-      </c>
+      <c r="A953"/>
       <c r="B953"/>
     </row>
     <row r="954">
@@ -8459,31 +8403,31 @@
     </row>
     <row r="967">
       <c r="A967" s="1" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
       <c r="B967" s="1" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
     </row>
     <row r="968">
       <c r="A968" s="1" t="s">
-        <v>520</v>
+        <v>512</v>
       </c>
       <c r="B968" s="1" t="s">
-        <v>521</v>
+        <v>513</v>
       </c>
     </row>
     <row r="969">
       <c r="A969" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B969" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="970">
       <c r="A970" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B970" s="2" t="s">
         <v>135</v>
@@ -8491,16 +8435,16 @@
     </row>
     <row r="971">
       <c r="A971" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="B971"/>
     </row>
     <row r="972">
       <c r="A972" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="B972" s="1" t="s">
-        <v>523</v>
+        <v>515</v>
       </c>
     </row>
     <row r="973">
@@ -8508,18 +8452,18 @@
         <v>7</v>
       </c>
       <c r="B973" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="974">
       <c r="A974"/>
       <c r="B974" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="975">
       <c r="A975" s="1" t="s">
-        <v>524</v>
+        <v>516</v>
       </c>
       <c r="B975" t="s">
         <v>249</v>
@@ -8527,15 +8471,15 @@
     </row>
     <row r="976">
       <c r="A976" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B976" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
     </row>
     <row r="977">
       <c r="A977" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B977" t="s">
         <v>224</v>
@@ -8551,7 +8495,7 @@
     </row>
     <row r="979">
       <c r="A979" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="B979"/>
     </row>
@@ -8560,7 +8504,7 @@
         <v>8</v>
       </c>
       <c r="B980" s="1" t="s">
-        <v>526</v>
+        <v>518</v>
       </c>
     </row>
     <row r="981">
@@ -8568,12 +8512,12 @@
         <v>29</v>
       </c>
       <c r="B981" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="982">
       <c r="A982" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="B982" s="2" t="s">
         <v>135</v>
@@ -8585,26 +8529,26 @@
     </row>
     <row r="984">
       <c r="A984" s="1" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="B984" s="1" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
     </row>
     <row r="985">
       <c r="A985" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B985" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="986">
       <c r="A986" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B986" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
     </row>
     <row r="987">
@@ -8612,7 +8556,7 @@
         <v>129</v>
       </c>
       <c r="B987" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
     </row>
     <row r="988">
@@ -8620,15 +8564,15 @@
         <v>116</v>
       </c>
       <c r="B988" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
     </row>
     <row r="989">
       <c r="A989" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
       <c r="B989" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
     </row>
     <row r="990">
@@ -8648,31 +8592,31 @@
     <row r="992">
       <c r="A992"/>
       <c r="B992" s="1" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
     </row>
     <row r="993">
       <c r="A993" s="1" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="B993" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="994">
       <c r="A994" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B994" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
     </row>
     <row r="995">
       <c r="A995" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B995" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="996">
@@ -8688,20 +8632,20 @@
         <v>29</v>
       </c>
       <c r="B997" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
     </row>
     <row r="998">
       <c r="A998" t="s">
-        <v>534</v>
+        <v>526</v>
       </c>
       <c r="B998" t="s">
-        <v>535</v>
+        <v>527</v>
       </c>
     </row>
     <row r="999">
       <c r="A999" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
       <c r="B999" t="s">
         <v>193</v>
@@ -8715,7 +8659,7 @@
     </row>
     <row r="1001">
       <c r="A1001" s="1" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="B1001" t="s">
         <v>165</v>
@@ -8723,7 +8667,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B1002" t="s">
         <v>205</v>
@@ -8745,13 +8689,13 @@
     </row>
     <row r="1005">
       <c r="A1005" s="1" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="B1005"/>
     </row>
     <row r="1006">
       <c r="A1006" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B1006"/>
     </row>
@@ -8769,7 +8713,7 @@
     </row>
     <row r="1009">
       <c r="A1009" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="B1009"/>
     </row>
@@ -8789,1008 +8733,968 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1">
-    <cfRule type="expression" dxfId="0" priority="210">
+    <cfRule type="expression" dxfId="0" priority="202">
       <formula>A1&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A2">
-    <cfRule type="expression" dxfId="0" priority="209">
+    <cfRule type="expression" dxfId="0" priority="201">
       <formula>A2&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A10:A10">
-    <cfRule type="expression" dxfId="0" priority="208">
+    <cfRule type="expression" dxfId="0" priority="200">
       <formula>A10&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20:A20">
-    <cfRule type="expression" dxfId="0" priority="207">
+    <cfRule type="expression" dxfId="0" priority="199">
       <formula>A20&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:A27">
-    <cfRule type="expression" dxfId="0" priority="206">
+    <cfRule type="expression" dxfId="0" priority="198">
       <formula>A27&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A47:A47">
-    <cfRule type="expression" dxfId="0" priority="205">
+    <cfRule type="expression" dxfId="0" priority="197">
       <formula>A47&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A48:A48">
-    <cfRule type="expression" dxfId="0" priority="204">
+    <cfRule type="expression" dxfId="0" priority="196">
       <formula>A48&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A60:A60">
-    <cfRule type="expression" dxfId="0" priority="203">
+    <cfRule type="expression" dxfId="0" priority="195">
       <formula>A60&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A67:A67">
-    <cfRule type="expression" dxfId="0" priority="202">
+    <cfRule type="expression" dxfId="0" priority="194">
       <formula>A67&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A78:A78">
-    <cfRule type="expression" dxfId="0" priority="201">
+    <cfRule type="expression" dxfId="0" priority="193">
       <formula>A78&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A93:A93">
-    <cfRule type="expression" dxfId="0" priority="200">
+    <cfRule type="expression" dxfId="0" priority="192">
       <formula>A93&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A94:A94">
-    <cfRule type="expression" dxfId="0" priority="199">
+    <cfRule type="expression" dxfId="0" priority="191">
       <formula>A94&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A103:A103">
-    <cfRule type="expression" dxfId="0" priority="198">
+    <cfRule type="expression" dxfId="0" priority="190">
       <formula>A103&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A109:A109">
-    <cfRule type="expression" dxfId="0" priority="197">
+    <cfRule type="expression" dxfId="0" priority="189">
       <formula>A109&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A117:A117">
-    <cfRule type="expression" dxfId="0" priority="196">
+    <cfRule type="expression" dxfId="0" priority="188">
       <formula>A117&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A125:A125">
-    <cfRule type="expression" dxfId="0" priority="195">
+    <cfRule type="expression" dxfId="0" priority="187">
       <formula>A125&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A139:A139">
-    <cfRule type="expression" dxfId="0" priority="194">
+    <cfRule type="expression" dxfId="0" priority="186">
       <formula>A139&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A140:A140">
-    <cfRule type="expression" dxfId="0" priority="193">
+    <cfRule type="expression" dxfId="0" priority="185">
       <formula>A140&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A144:A144">
-    <cfRule type="expression" dxfId="0" priority="192">
+    <cfRule type="expression" dxfId="0" priority="184">
       <formula>A144&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A185:A185">
-    <cfRule type="expression" dxfId="1" priority="191">
+    <cfRule type="expression" dxfId="1" priority="183">
       <formula>A185&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A186:A186">
-    <cfRule type="expression" dxfId="1" priority="190">
+    <cfRule type="expression" dxfId="1" priority="182">
       <formula>A186&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A194:A194">
-    <cfRule type="expression" dxfId="1" priority="189">
+    <cfRule type="expression" dxfId="1" priority="181">
       <formula>A194&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A205:A205">
-    <cfRule type="expression" dxfId="1" priority="188">
+    <cfRule type="expression" dxfId="1" priority="180">
       <formula>A205&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A214:A214">
-    <cfRule type="expression" dxfId="1" priority="187">
+    <cfRule type="expression" dxfId="1" priority="179">
       <formula>A214&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A231:A231">
-    <cfRule type="expression" dxfId="1" priority="186">
+    <cfRule type="expression" dxfId="1" priority="178">
       <formula>A231&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A232:A232">
-    <cfRule type="expression" dxfId="1" priority="185">
+    <cfRule type="expression" dxfId="1" priority="177">
       <formula>A232&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A242:A242">
-    <cfRule type="expression" dxfId="1" priority="184">
+    <cfRule type="expression" dxfId="1" priority="176">
       <formula>A242&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A260:A260">
-    <cfRule type="expression" dxfId="1" priority="183">
+    <cfRule type="expression" dxfId="1" priority="175">
       <formula>A260&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A277:A277">
-    <cfRule type="expression" dxfId="1" priority="182">
+    <cfRule type="expression" dxfId="1" priority="174">
       <formula>A277&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A278:A278">
-    <cfRule type="expression" dxfId="1" priority="181">
+    <cfRule type="expression" dxfId="1" priority="173">
       <formula>A278&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A298:A298">
-    <cfRule type="expression" dxfId="1" priority="180">
+    <cfRule type="expression" dxfId="1" priority="172">
       <formula>A298&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A308:A308">
-    <cfRule type="expression" dxfId="1" priority="179">
+    <cfRule type="expression" dxfId="1" priority="171">
       <formula>A308&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A313:A313">
-    <cfRule type="expression" dxfId="1" priority="178">
+    <cfRule type="expression" dxfId="1" priority="170">
       <formula>A313&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A323:A323">
-    <cfRule type="expression" dxfId="1" priority="177">
+    <cfRule type="expression" dxfId="1" priority="169">
       <formula>A323&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A324:A324">
-    <cfRule type="expression" dxfId="1" priority="176">
+    <cfRule type="expression" dxfId="1" priority="168">
       <formula>A324&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A328:A328">
-    <cfRule type="expression" dxfId="1" priority="175">
+    <cfRule type="expression" dxfId="1" priority="167">
       <formula>A328&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A369:A369">
-    <cfRule type="expression" dxfId="2" priority="174">
+    <cfRule type="expression" dxfId="2" priority="166">
       <formula>A369&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A370:A370">
-    <cfRule type="expression" dxfId="2" priority="173">
+    <cfRule type="expression" dxfId="2" priority="165">
       <formula>A370&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A380:A380">
-    <cfRule type="expression" dxfId="2" priority="172">
+    <cfRule type="expression" dxfId="2" priority="164">
       <formula>A380&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A392:A392">
-    <cfRule type="expression" dxfId="2" priority="171">
+    <cfRule type="expression" dxfId="2" priority="163">
       <formula>A392&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A415:A415">
-    <cfRule type="expression" dxfId="2" priority="170">
+    <cfRule type="expression" dxfId="2" priority="162">
       <formula>A415&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A416:A416">
-    <cfRule type="expression" dxfId="2" priority="169">
+    <cfRule type="expression" dxfId="2" priority="161">
       <formula>A416&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A427:A427">
-    <cfRule type="expression" dxfId="2" priority="168">
+    <cfRule type="expression" dxfId="2" priority="160">
       <formula>A427&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A439:A439">
-    <cfRule type="expression" dxfId="2" priority="167">
+    <cfRule type="expression" dxfId="2" priority="159">
       <formula>A439&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A449:A449">
-    <cfRule type="expression" dxfId="2" priority="166">
+    <cfRule type="expression" dxfId="2" priority="158">
       <formula>A449&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A461:A461">
-    <cfRule type="expression" dxfId="2" priority="165">
+    <cfRule type="expression" dxfId="2" priority="157">
       <formula>A461&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A462:A462">
-    <cfRule type="expression" dxfId="2" priority="164">
+    <cfRule type="expression" dxfId="2" priority="156">
       <formula>A462&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A472:A472">
-    <cfRule type="expression" dxfId="2" priority="163">
+    <cfRule type="expression" dxfId="2" priority="155">
       <formula>A472&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A482:A482">
-    <cfRule type="expression" dxfId="2" priority="162">
+    <cfRule type="expression" dxfId="2" priority="154">
       <formula>A482&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A492:A492">
-    <cfRule type="expression" dxfId="2" priority="161">
+    <cfRule type="expression" dxfId="2" priority="153">
       <formula>A492&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A507:A507">
-    <cfRule type="expression" dxfId="2" priority="160">
+    <cfRule type="expression" dxfId="2" priority="152">
       <formula>A507&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A508:A508">
-    <cfRule type="expression" dxfId="2" priority="159">
+    <cfRule type="expression" dxfId="2" priority="151">
       <formula>A508&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A518:A518">
-    <cfRule type="expression" dxfId="2" priority="158">
-      <formula>A518&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A521:A521">
-    <cfRule type="expression" dxfId="2" priority="157">
-      <formula>A521&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A525:A525">
-    <cfRule type="expression" dxfId="2" priority="156">
-      <formula>A525&lt;&gt;0</formula>
+  <conditionalFormatting sqref="A516:A516">
+    <cfRule type="expression" dxfId="2" priority="150">
+      <formula>A516&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A553:A553">
-    <cfRule type="expression" dxfId="3" priority="155">
+    <cfRule type="expression" dxfId="3" priority="149">
       <formula>A553&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A554:A554">
-    <cfRule type="expression" dxfId="3" priority="154">
+    <cfRule type="expression" dxfId="3" priority="148">
       <formula>A554&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A558:A558">
-    <cfRule type="expression" dxfId="3" priority="153">
+    <cfRule type="expression" dxfId="3" priority="147">
       <formula>A558&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A566:A566">
-    <cfRule type="expression" dxfId="3" priority="152">
+    <cfRule type="expression" dxfId="3" priority="146">
       <formula>A566&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A599:A599">
-    <cfRule type="expression" dxfId="4" priority="151">
+    <cfRule type="expression" dxfId="4" priority="145">
       <formula>A599&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A600:A600">
-    <cfRule type="expression" dxfId="4" priority="150">
+    <cfRule type="expression" dxfId="4" priority="144">
       <formula>A600&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A608:A608">
-    <cfRule type="expression" dxfId="4" priority="149">
+    <cfRule type="expression" dxfId="4" priority="143">
       <formula>A608&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A617:A617">
-    <cfRule type="expression" dxfId="4" priority="148">
+    <cfRule type="expression" dxfId="4" priority="142">
       <formula>A617&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A626:A626">
-    <cfRule type="expression" dxfId="4" priority="147">
+    <cfRule type="expression" dxfId="4" priority="141">
       <formula>A626&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A631:A631">
-    <cfRule type="expression" dxfId="4" priority="146">
+    <cfRule type="expression" dxfId="4" priority="140">
       <formula>A631&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A645:A645">
-    <cfRule type="expression" dxfId="4" priority="145">
+    <cfRule type="expression" dxfId="4" priority="139">
       <formula>A645&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A646:A646">
-    <cfRule type="expression" dxfId="4" priority="144">
+    <cfRule type="expression" dxfId="4" priority="138">
       <formula>A646&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A653:A653">
-    <cfRule type="expression" dxfId="4" priority="143">
+    <cfRule type="expression" dxfId="4" priority="137">
       <formula>A653&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A661:A661">
-    <cfRule type="expression" dxfId="4" priority="142">
+    <cfRule type="expression" dxfId="4" priority="136">
       <formula>A661&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A668:A668">
-    <cfRule type="expression" dxfId="4" priority="141">
+    <cfRule type="expression" dxfId="4" priority="135">
       <formula>A668&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A672:A672">
-    <cfRule type="expression" dxfId="4" priority="140">
+    <cfRule type="expression" dxfId="4" priority="134">
       <formula>A672&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A680:A680">
-    <cfRule type="expression" dxfId="4" priority="139">
+    <cfRule type="expression" dxfId="4" priority="133">
       <formula>A680&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A684:A684">
-    <cfRule type="expression" dxfId="4" priority="138">
+    <cfRule type="expression" dxfId="4" priority="132">
       <formula>A684&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A691:A691">
-    <cfRule type="expression" dxfId="4" priority="137">
+    <cfRule type="expression" dxfId="4" priority="131">
       <formula>A691&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A692:A692">
-    <cfRule type="expression" dxfId="4" priority="136">
+    <cfRule type="expression" dxfId="4" priority="130">
       <formula>A692&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A699:A699">
-    <cfRule type="expression" dxfId="4" priority="135">
+    <cfRule type="expression" dxfId="4" priority="129">
       <formula>A699&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A707:A707">
-    <cfRule type="expression" dxfId="4" priority="134">
+    <cfRule type="expression" dxfId="4" priority="128">
       <formula>A707&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A737:A737">
-    <cfRule type="expression" dxfId="5" priority="133">
+    <cfRule type="expression" dxfId="5" priority="127">
       <formula>A737&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A738:A738">
-    <cfRule type="expression" dxfId="5" priority="132">
+    <cfRule type="expression" dxfId="5" priority="126">
       <formula>A738&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A748:A748">
-    <cfRule type="expression" dxfId="5" priority="131">
+    <cfRule type="expression" dxfId="5" priority="125">
       <formula>A748&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A761:A761">
-    <cfRule type="expression" dxfId="5" priority="130">
+    <cfRule type="expression" dxfId="5" priority="124">
       <formula>A761&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A770:A770">
-    <cfRule type="expression" dxfId="5" priority="129">
+    <cfRule type="expression" dxfId="5" priority="123">
       <formula>A770&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A783:A783">
-    <cfRule type="expression" dxfId="5" priority="128">
+    <cfRule type="expression" dxfId="5" priority="122">
       <formula>A783&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A784:A784">
-    <cfRule type="expression" dxfId="5" priority="127">
+    <cfRule type="expression" dxfId="5" priority="121">
       <formula>A784&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A795:A795">
-    <cfRule type="expression" dxfId="5" priority="126">
+    <cfRule type="expression" dxfId="5" priority="120">
       <formula>A795&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A804:A804">
-    <cfRule type="expression" dxfId="5" priority="125">
+    <cfRule type="expression" dxfId="5" priority="119">
       <formula>A804&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A813:A813">
-    <cfRule type="expression" dxfId="5" priority="124">
+    <cfRule type="expression" dxfId="5" priority="118">
       <formula>A813&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A829:A829">
-    <cfRule type="expression" dxfId="5" priority="123">
+    <cfRule type="expression" dxfId="5" priority="117">
       <formula>A829&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A830:A830">
-    <cfRule type="expression" dxfId="5" priority="122">
+    <cfRule type="expression" dxfId="5" priority="116">
       <formula>A830&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A840:A840">
-    <cfRule type="expression" dxfId="5" priority="121">
+    <cfRule type="expression" dxfId="5" priority="115">
       <formula>A840&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A853:A853">
-    <cfRule type="expression" dxfId="5" priority="120">
+    <cfRule type="expression" dxfId="5" priority="114">
       <formula>A853&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A875:A875">
-    <cfRule type="expression" dxfId="6" priority="119">
+    <cfRule type="expression" dxfId="6" priority="113">
       <formula>A875&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A876:A876">
-    <cfRule type="expression" dxfId="6" priority="118">
+    <cfRule type="expression" dxfId="6" priority="112">
       <formula>A876&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A886:A886">
-    <cfRule type="expression" dxfId="6" priority="117">
+    <cfRule type="expression" dxfId="6" priority="111">
       <formula>A886&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A889:A889">
-    <cfRule type="expression" dxfId="6" priority="116">
-      <formula>A889&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A895:A895">
-    <cfRule type="expression" dxfId="6" priority="115">
-      <formula>A895&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A904:A904">
-    <cfRule type="expression" dxfId="6" priority="114">
-      <formula>A904&lt;&gt;0</formula>
+  <conditionalFormatting sqref="A892:A892">
+    <cfRule type="expression" dxfId="6" priority="110">
+      <formula>A892&lt;&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A901:A901">
+    <cfRule type="expression" dxfId="6" priority="109">
+      <formula>A901&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A921:A921">
-    <cfRule type="expression" dxfId="6" priority="113">
+    <cfRule type="expression" dxfId="6" priority="108">
       <formula>A921&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A922:A922">
-    <cfRule type="expression" dxfId="6" priority="112">
+    <cfRule type="expression" dxfId="6" priority="107">
       <formula>A922&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A932:A932">
-    <cfRule type="expression" dxfId="6" priority="111">
+    <cfRule type="expression" dxfId="6" priority="106">
       <formula>A932&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A945:A945">
-    <cfRule type="expression" dxfId="6" priority="110">
-      <formula>A945&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A967:A967">
-    <cfRule type="expression" dxfId="7" priority="109">
+    <cfRule type="expression" dxfId="7" priority="105">
       <formula>A967&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A968:A968">
-    <cfRule type="expression" dxfId="7" priority="108">
+    <cfRule type="expression" dxfId="7" priority="104">
       <formula>A968&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A975:A975">
-    <cfRule type="expression" dxfId="7" priority="107">
+    <cfRule type="expression" dxfId="7" priority="103">
       <formula>A975&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A984:A984">
-    <cfRule type="expression" dxfId="7" priority="106">
+    <cfRule type="expression" dxfId="7" priority="102">
       <formula>A984&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A993:A993">
-    <cfRule type="expression" dxfId="7" priority="105">
+    <cfRule type="expression" dxfId="7" priority="101">
       <formula>A993&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1001:A1001">
-    <cfRule type="expression" dxfId="7" priority="104">
+    <cfRule type="expression" dxfId="7" priority="100">
       <formula>A1001&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1005:A1005">
-    <cfRule type="expression" dxfId="7" priority="103">
+    <cfRule type="expression" dxfId="7" priority="99">
       <formula>A1005&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1">
-    <cfRule type="expression" dxfId="0" priority="102">
+    <cfRule type="expression" dxfId="0" priority="98">
       <formula>B1&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B2">
-    <cfRule type="expression" dxfId="0" priority="101">
+    <cfRule type="expression" dxfId="0" priority="97">
       <formula>B2&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:B14">
-    <cfRule type="expression" dxfId="0" priority="100">
+    <cfRule type="expression" dxfId="0" priority="96">
       <formula>B14&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:B32">
-    <cfRule type="expression" dxfId="0" priority="99">
+    <cfRule type="expression" dxfId="0" priority="95">
       <formula>B32&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B47:B47">
-    <cfRule type="expression" dxfId="0" priority="98">
+    <cfRule type="expression" dxfId="0" priority="94">
       <formula>B47&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B48:B48">
-    <cfRule type="expression" dxfId="0" priority="97">
+    <cfRule type="expression" dxfId="0" priority="93">
       <formula>B48&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B64:B64">
-    <cfRule type="expression" dxfId="0" priority="96">
+    <cfRule type="expression" dxfId="0" priority="92">
       <formula>B64&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B76:B76">
-    <cfRule type="expression" dxfId="0" priority="95">
+    <cfRule type="expression" dxfId="0" priority="91">
       <formula>B76&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93:B93">
-    <cfRule type="expression" dxfId="0" priority="94">
+    <cfRule type="expression" dxfId="0" priority="90">
       <formula>B93&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B94:B94">
-    <cfRule type="expression" dxfId="0" priority="93">
+    <cfRule type="expression" dxfId="0" priority="89">
       <formula>B94&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B105:B105">
-    <cfRule type="expression" dxfId="0" priority="92">
+    <cfRule type="expression" dxfId="0" priority="88">
       <formula>B105&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B118:B118">
-    <cfRule type="expression" dxfId="0" priority="91">
+    <cfRule type="expression" dxfId="0" priority="87">
       <formula>B118&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B129:B129">
-    <cfRule type="expression" dxfId="0" priority="90">
+    <cfRule type="expression" dxfId="0" priority="86">
       <formula>B129&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B139:B139">
-    <cfRule type="expression" dxfId="0" priority="89">
+    <cfRule type="expression" dxfId="0" priority="85">
       <formula>B139&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B140:B140">
-    <cfRule type="expression" dxfId="0" priority="88">
+    <cfRule type="expression" dxfId="0" priority="84">
       <formula>B140&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B185:B185">
-    <cfRule type="expression" dxfId="1" priority="87">
+    <cfRule type="expression" dxfId="1" priority="83">
       <formula>B185&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B186:B186">
-    <cfRule type="expression" dxfId="1" priority="86">
+    <cfRule type="expression" dxfId="1" priority="82">
       <formula>B186&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B195:B195">
-    <cfRule type="expression" dxfId="1" priority="85">
+    <cfRule type="expression" dxfId="1" priority="81">
       <formula>B195&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B205:B205">
-    <cfRule type="expression" dxfId="1" priority="84">
+    <cfRule type="expression" dxfId="1" priority="80">
       <formula>B205&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B214:B214">
-    <cfRule type="expression" dxfId="1" priority="83">
+    <cfRule type="expression" dxfId="1" priority="79">
       <formula>B214&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B231:B231">
-    <cfRule type="expression" dxfId="1" priority="82">
+    <cfRule type="expression" dxfId="1" priority="78">
       <formula>B231&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B232:B232">
-    <cfRule type="expression" dxfId="1" priority="81">
+    <cfRule type="expression" dxfId="1" priority="77">
       <formula>B232&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B242:B242">
-    <cfRule type="expression" dxfId="1" priority="80">
+    <cfRule type="expression" dxfId="1" priority="76">
       <formula>B242&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B250:B250">
-    <cfRule type="expression" dxfId="1" priority="79">
+    <cfRule type="expression" dxfId="1" priority="75">
       <formula>B250&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B277:B277">
-    <cfRule type="expression" dxfId="1" priority="78">
+    <cfRule type="expression" dxfId="1" priority="74">
       <formula>B277&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B278:B278">
-    <cfRule type="expression" dxfId="1" priority="77">
+    <cfRule type="expression" dxfId="1" priority="73">
       <formula>B278&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B290:B290">
-    <cfRule type="expression" dxfId="1" priority="76">
+    <cfRule type="expression" dxfId="1" priority="72">
       <formula>B290&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B301:B301">
-    <cfRule type="expression" dxfId="1" priority="75">
+    <cfRule type="expression" dxfId="1" priority="71">
       <formula>B301&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B305:B305">
-    <cfRule type="expression" dxfId="1" priority="74">
+    <cfRule type="expression" dxfId="1" priority="70">
       <formula>B305&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B315:B315">
-    <cfRule type="expression" dxfId="1" priority="73">
+    <cfRule type="expression" dxfId="1" priority="69">
       <formula>B315&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B323:B323">
-    <cfRule type="expression" dxfId="1" priority="72">
+    <cfRule type="expression" dxfId="1" priority="68">
       <formula>B323&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B324:B324">
-    <cfRule type="expression" dxfId="1" priority="71">
+    <cfRule type="expression" dxfId="1" priority="67">
       <formula>B324&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B328:B328">
-    <cfRule type="expression" dxfId="1" priority="70">
+    <cfRule type="expression" dxfId="1" priority="66">
       <formula>B328&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B369:B369">
-    <cfRule type="expression" dxfId="2" priority="69">
+    <cfRule type="expression" dxfId="2" priority="65">
       <formula>B369&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B370:B370">
-    <cfRule type="expression" dxfId="2" priority="68">
+    <cfRule type="expression" dxfId="2" priority="64">
       <formula>B370&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B381:B381">
-    <cfRule type="expression" dxfId="2" priority="67">
+    <cfRule type="expression" dxfId="2" priority="63">
       <formula>B381&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B393:B393">
-    <cfRule type="expression" dxfId="2" priority="66">
+    <cfRule type="expression" dxfId="2" priority="62">
       <formula>B393&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B415:B415">
-    <cfRule type="expression" dxfId="2" priority="65">
+    <cfRule type="expression" dxfId="2" priority="61">
       <formula>B415&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B416:B416">
-    <cfRule type="expression" dxfId="2" priority="64">
+    <cfRule type="expression" dxfId="2" priority="60">
       <formula>B416&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B428:B428">
-    <cfRule type="expression" dxfId="2" priority="63">
+    <cfRule type="expression" dxfId="2" priority="59">
       <formula>B428&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B440:B440">
-    <cfRule type="expression" dxfId="2" priority="62">
+    <cfRule type="expression" dxfId="2" priority="58">
       <formula>B440&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B449:B449">
-    <cfRule type="expression" dxfId="2" priority="61">
+    <cfRule type="expression" dxfId="2" priority="57">
       <formula>B449&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B461:B461">
-    <cfRule type="expression" dxfId="2" priority="60">
+    <cfRule type="expression" dxfId="2" priority="56">
       <formula>B461&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B462:B462">
-    <cfRule type="expression" dxfId="2" priority="59">
+    <cfRule type="expression" dxfId="2" priority="55">
       <formula>B462&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B469:B469">
-    <cfRule type="expression" dxfId="2" priority="58">
+    <cfRule type="expression" dxfId="2" priority="54">
       <formula>B469&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B480:B480">
-    <cfRule type="expression" dxfId="2" priority="57">
+    <cfRule type="expression" dxfId="2" priority="53">
       <formula>B480&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B491:B491">
-    <cfRule type="expression" dxfId="2" priority="56">
+    <cfRule type="expression" dxfId="2" priority="52">
       <formula>B491&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B494:B494">
-    <cfRule type="expression" dxfId="2" priority="55">
-      <formula>B494&lt;&gt;0</formula>
+  <conditionalFormatting sqref="B496:B496">
+    <cfRule type="expression" dxfId="2" priority="51">
+      <formula>B496&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B507:B507">
-    <cfRule type="expression" dxfId="2" priority="54">
+    <cfRule type="expression" dxfId="2" priority="50">
       <formula>B507&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B508:B508">
-    <cfRule type="expression" dxfId="2" priority="53">
+    <cfRule type="expression" dxfId="2" priority="49">
       <formula>B508&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B511:B511">
-    <cfRule type="expression" dxfId="2" priority="52">
-      <formula>B511&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B519:B519">
-    <cfRule type="expression" dxfId="2" priority="51">
-      <formula>B519&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B522:B522">
-    <cfRule type="expression" dxfId="2" priority="50">
-      <formula>B522&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B553:B553">
-    <cfRule type="expression" dxfId="3" priority="49">
+    <cfRule type="expression" dxfId="3" priority="48">
       <formula>B553&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B554:B554">
-    <cfRule type="expression" dxfId="3" priority="48">
+    <cfRule type="expression" dxfId="3" priority="47">
       <formula>B554&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B560:B560">
-    <cfRule type="expression" dxfId="3" priority="47">
+    <cfRule type="expression" dxfId="3" priority="46">
       <formula>B560&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B570:B570">
-    <cfRule type="expression" dxfId="3" priority="46">
+    <cfRule type="expression" dxfId="3" priority="45">
       <formula>B570&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B599:B599">
-    <cfRule type="expression" dxfId="4" priority="45">
+    <cfRule type="expression" dxfId="4" priority="44">
       <formula>B599&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B600:B600">
-    <cfRule type="expression" dxfId="4" priority="44">
+    <cfRule type="expression" dxfId="4" priority="43">
       <formula>B600&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B608:B608">
-    <cfRule type="expression" dxfId="4" priority="43">
+    <cfRule type="expression" dxfId="4" priority="42">
       <formula>B608&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B615:B615">
-    <cfRule type="expression" dxfId="4" priority="42">
+    <cfRule type="expression" dxfId="4" priority="41">
       <formula>B615&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B624:B624">
-    <cfRule type="expression" dxfId="4" priority="41">
+    <cfRule type="expression" dxfId="4" priority="40">
       <formula>B624&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B632:B632">
-    <cfRule type="expression" dxfId="4" priority="40">
+    <cfRule type="expression" dxfId="4" priority="39">
       <formula>B632&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B645:B645">
-    <cfRule type="expression" dxfId="4" priority="39">
+    <cfRule type="expression" dxfId="4" priority="38">
       <formula>B645&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B646:B646">
-    <cfRule type="expression" dxfId="4" priority="38">
+    <cfRule type="expression" dxfId="4" priority="37">
       <formula>B646&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B654:B654">
-    <cfRule type="expression" dxfId="4" priority="37">
+    <cfRule type="expression" dxfId="4" priority="36">
       <formula>B654&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B663:B663">
-    <cfRule type="expression" dxfId="4" priority="36">
+    <cfRule type="expression" dxfId="4" priority="35">
       <formula>B663&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B670:B670">
-    <cfRule type="expression" dxfId="4" priority="35">
+    <cfRule type="expression" dxfId="4" priority="34">
       <formula>B670&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B679:B679">
-    <cfRule type="expression" dxfId="4" priority="34">
+    <cfRule type="expression" dxfId="4" priority="33">
       <formula>B679&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B683:B683">
-    <cfRule type="expression" dxfId="4" priority="33">
+    <cfRule type="expression" dxfId="4" priority="32">
       <formula>B683&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B691:B691">
-    <cfRule type="expression" dxfId="4" priority="32">
+    <cfRule type="expression" dxfId="4" priority="31">
       <formula>B691&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B692:B692">
-    <cfRule type="expression" dxfId="4" priority="31">
+    <cfRule type="expression" dxfId="4" priority="30">
       <formula>B692&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B702:B702">
-    <cfRule type="expression" dxfId="4" priority="30">
+    <cfRule type="expression" dxfId="4" priority="29">
       <formula>B702&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B706:B706">
-    <cfRule type="expression" dxfId="4" priority="29">
+    <cfRule type="expression" dxfId="4" priority="28">
       <formula>B706&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B737:B737">
-    <cfRule type="expression" dxfId="5" priority="28">
+    <cfRule type="expression" dxfId="5" priority="27">
       <formula>B737&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B738:B738">
-    <cfRule type="expression" dxfId="5" priority="27">
+    <cfRule type="expression" dxfId="5" priority="26">
       <formula>B738&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B747:B747">
-    <cfRule type="expression" dxfId="5" priority="26">
+    <cfRule type="expression" dxfId="5" priority="25">
       <formula>B747&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B757:B757">
-    <cfRule type="expression" dxfId="5" priority="25">
+    <cfRule type="expression" dxfId="5" priority="24">
       <formula>B757&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B766:B766">
-    <cfRule type="expression" dxfId="5" priority="24">
+    <cfRule type="expression" dxfId="5" priority="23">
       <formula>B766&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B783:B783">
-    <cfRule type="expression" dxfId="5" priority="23">
+    <cfRule type="expression" dxfId="5" priority="22">
       <formula>B783&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B784:B784">
-    <cfRule type="expression" dxfId="5" priority="22">
+    <cfRule type="expression" dxfId="5" priority="21">
       <formula>B784&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B794:B794">
-    <cfRule type="expression" dxfId="5" priority="21">
+    <cfRule type="expression" dxfId="5" priority="20">
       <formula>B794&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B804:B804">
-    <cfRule type="expression" dxfId="5" priority="20">
+    <cfRule type="expression" dxfId="5" priority="19">
       <formula>B804&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B811:B811">
-    <cfRule type="expression" dxfId="5" priority="19">
+    <cfRule type="expression" dxfId="5" priority="18">
       <formula>B811&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B829:B829">
-    <cfRule type="expression" dxfId="5" priority="18">
+    <cfRule type="expression" dxfId="5" priority="17">
       <formula>B829&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B830:B830">
-    <cfRule type="expression" dxfId="5" priority="17">
+    <cfRule type="expression" dxfId="5" priority="16">
       <formula>B830&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B840:B840">
-    <cfRule type="expression" dxfId="5" priority="16">
+    <cfRule type="expression" dxfId="5" priority="15">
       <formula>B840&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B875:B875">
-    <cfRule type="expression" dxfId="6" priority="15">
+    <cfRule type="expression" dxfId="6" priority="14">
       <formula>B875&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B876:B876">
-    <cfRule type="expression" dxfId="6" priority="14">
+    <cfRule type="expression" dxfId="6" priority="13">
       <formula>B876&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B884:B884">
-    <cfRule type="expression" dxfId="6" priority="13">
+    <cfRule type="expression" dxfId="6" priority="12">
       <formula>B884&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B887:B887">
-    <cfRule type="expression" dxfId="6" priority="12">
-      <formula>B887&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B898:B898">
+  <conditionalFormatting sqref="B895:B895">
     <cfRule type="expression" dxfId="6" priority="11">
-      <formula>B898&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B909:B909">
+      <formula>B895&lt;&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B906:B906">
     <cfRule type="expression" dxfId="6" priority="10">
-      <formula>B909&lt;&gt;0</formula>
+      <formula>B906&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B921:B921">
@@ -9803,9 +9707,9 @@
       <formula>B922&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B925:B925">
+  <conditionalFormatting sqref="B935:B935">
     <cfRule type="expression" dxfId="6" priority="7">
-      <formula>B925&lt;&gt;0</formula>
+      <formula>B935&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B967:B967">

</xml_diff>